<commit_message>
Remove past report HTMLs from tracking
</commit_message>
<xml_diff>
--- a/data_xlsx_archive/志明AI實驗數據_6_1-6_15.xlsx
+++ b/data_xlsx_archive/志明AI實驗數據_6_1-6_15.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -1739,7 +1739,7 @@
         <v>期間</v>
       </c>
       <c r="B6" t="str">
-        <v>2026/6/1 – 6/12</v>
+        <v>2026/6/1 – 6/15</v>
       </c>
     </row>
     <row r="7">
@@ -1747,7 +1747,7 @@
         <v>總組數</v>
       </c>
       <c r="B7" t="str">
-        <v>25 組（跨型態 19、文案 5、其他 1）</v>
+        <v>28 組（跨型態 22、文案 5、其他 1）</v>
       </c>
     </row>
     <row r="8">

</xml_diff>